<commit_message>
refactor: make spreadsheet imports text only
</commit_message>
<xml_diff>
--- a/public/题库模板.xlsx
+++ b/public/题库模板.xlsx
@@ -398,12 +398,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:L5"/>
   <cols>
     <col min="1" max="1" width="46.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="42.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
     <col min="5" max="5" width="22.83203125" customWidth="1"/>
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
     <col min="7" max="7" width="22.83203125" customWidth="1"/>
@@ -412,7 +412,6 @@
     <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="22.83203125" customWidth="1"/>
     <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,33 +425,30 @@
         <v>答案</v>
       </c>
       <c r="D1" t="str">
-        <v>图片地址</v>
+        <v>标签</v>
       </c>
       <c r="E1" t="str">
-        <v>标签</v>
+        <v>A</v>
       </c>
       <c r="F1" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="G1" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="H1" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="I1" t="str">
-        <v>D</v>
+        <v>E</v>
       </c>
       <c r="J1" t="str">
-        <v>E</v>
+        <v>F</v>
       </c>
       <c r="K1" t="str">
-        <v>F</v>
+        <v>G</v>
       </c>
       <c r="L1" t="str">
-        <v>G</v>
-      </c>
-      <c r="M1" t="str">
         <v>H</v>
       </c>
     </row>
@@ -467,21 +463,18 @@
         <v>A</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>基础，示例</v>
       </c>
       <c r="E2" t="str">
-        <v>基础，示例</v>
+        <v>传输电能</v>
       </c>
       <c r="F2" t="str">
-        <v>传输电能</v>
+        <v>装饰线路</v>
       </c>
       <c r="G2" t="str">
-        <v>装饰线路</v>
+        <v>储存电能</v>
       </c>
       <c r="H2" t="str">
-        <v>储存电能</v>
-      </c>
-      <c r="I2" t="str">
         <v>测量温度</v>
       </c>
     </row>
@@ -496,21 +489,18 @@
         <v>AB</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>安全，示例</v>
       </c>
       <c r="E3" t="str">
-        <v>安全，示例</v>
+        <v>佩戴防护用品</v>
       </c>
       <c r="F3" t="str">
-        <v>佩戴防护用品</v>
+        <v>核对线路编号</v>
       </c>
       <c r="G3" t="str">
-        <v>核对线路编号</v>
+        <v>跨越警戒区域</v>
       </c>
       <c r="H3" t="str">
-        <v>跨越警戒区域</v>
-      </c>
-      <c r="I3" t="str">
         <v>跳过危险点记录</v>
       </c>
     </row>
@@ -525,15 +515,12 @@
         <v>A</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>安全，示例</v>
       </c>
       <c r="E4" t="str">
-        <v>安全，示例</v>
+        <v>正确</v>
       </c>
       <c r="F4" t="str">
-        <v>正确</v>
-      </c>
-      <c r="G4" t="str">
         <v>错误</v>
       </c>
     </row>
@@ -548,22 +535,19 @@
         <v>12.5</v>
       </c>
       <c r="D5" t="str">
-        <v>https://example.com/question.png</v>
-      </c>
-      <c r="E5" t="str">
         <v>计算，示例</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B12"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="110.83203125" customWidth="1"/>
@@ -616,63 +600,55 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>图片地址</v>
+        <v>标签</v>
       </c>
       <c r="B7" t="str">
-        <v>可选。填写完整的 http/https 图片 URL；导入后显示在题干下方。请确保各设备都能访问该地址。</v>
+        <v>可选。多个标签使用中文逗号、英文逗号或顿号分隔。</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>标签</v>
+        <v>选项</v>
       </c>
       <c r="B8" t="str">
-        <v>可选。多个标签使用中文逗号、英文逗号或顿号分隔。</v>
+        <v>单选、多选、判断题从 A 列开始连续填写，不得断列；判断题必须依次为“正确、错误”。计算题不要填写选项。</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>选项</v>
+        <v>计算题误差</v>
       </c>
       <c r="B9" t="str">
-        <v>单选、多选、判断题从 A 列开始连续填写，不得断列；判断题必须依次为“正确、错误”。计算题不要填写选项。</v>
+        <v>计算题按配置页中的“计算题允许误差”判定，使用相对误差百分比；标准答案为 0 时按同一百分比折算为绝对误差。</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>计算题误差</v>
+        <v>图片题</v>
       </c>
       <c r="B10" t="str">
-        <v>计算题按配置页中的“计算题允许误差”判定，使用相对误差百分比；标准答案为 0 时按同一百分比折算为绝对误差。</v>
+        <v>Excel 只导入纯文字题。导入后请在题目编辑器中选择本机图片并插入到题干或选项的任意位置；图片会作为私有资产同步。</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>图片与离线</v>
+        <v>限制</v>
       </c>
       <c r="B11" t="str">
-        <v>图片 URL 由浏览器加载；题目文字和学习记录仍保存在本机并通过 Sync v5 同步。</v>
+        <v>单次最多导入 20,000 题；每题最多 24 个选项；Excel 文件最大 12 MB。</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>限制</v>
+        <v>安全提醒</v>
       </c>
       <c r="B12" t="str">
-        <v>单次最多导入 20,000 题；每题最多 24 个选项；Excel 文件最大 12 MB。</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>安全提醒</v>
-      </c>
-      <c r="B13" t="str">
         <v>不要在工作簿中填写 GitHub 令牌或其他账号凭据。</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: refresh Excel template for all question types
* fix: align xlsx template with all question types

* fix: publish refreshed xlsx template

* fix: keep xlsx template compact

* test: lock compact xlsx template contract

* ci: regenerate xlsx template for verification

* ci: persist regenerated xlsx template once

* ci: checkout pr head for template persistence

* chore: regenerate xlsx template

* ci: restore pull request checks

---------

Co-authored-by: github-actions[bot] <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/题库模板.xlsx
+++ b/public/题库模板.xlsx
@@ -51,17 +51,11 @@
     <col min="4" max="4" width="34" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
-    <col min="14" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="22" customWidth="1"/>
-    <col min="16" max="16" width="22" customWidth="1"/>
-    <col min="17" max="17" width="28" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -97,55 +91,25 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>答案3</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>答案4</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
         <is>
           <t>图片1</t>
         </is>
@@ -177,22 +141,22 @@
           <t>A</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>传输电能</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>装饰线路</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>传输电能</t>
+          <t>储存电能</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
-        <is>
-          <t>装饰线路</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>储存电能</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
         <is>
           <t>测量温度</t>
         </is>
@@ -224,22 +188,22 @@
           <t>AB</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>佩戴防护用品</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>核对线路编号</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>佩戴防护用品</t>
+          <t>跨越警戒区域</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
-        <is>
-          <t>核对线路编号</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>跨越警戒区域</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
         <is>
           <t>跳过危险点记录</t>
         </is>
@@ -271,12 +235,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>正确</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>错误</t>
         </is>
@@ -367,29 +331,115 @@
           <t>A</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>拾卷</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>浏览器</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>拾卷</t>
+          <t>相册</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>浏览器</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>相册</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
           <t>日历</t>
         </is>
       </c>
-      <c r="Q7" t="str">
+      <c r="K7" t="str">
         <f>_xlfn.DISPIMG("ID_TEMPLATE_SHIJUAN_APP_ICON",1)</f>
         <v>=DISPIMG("ID_TEMPLATE_SHIJUAN_APP_ICON",1)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>示例·单空填空（填好后删）输电线路的主要作用是【空1】。</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>填空</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>填空，示例</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>示例解析：同一空允许多个等价答案时，在答案单元格内用 || 分隔。</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>传输电能||输送电能</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>示例·多空填空（填好后删）三相交流电中，相邻两相电动势的相位差为【空1】°，我国电力系统工频为【空2】Hz。</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>填空</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>填空，多空，示例</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>示例解析：答案1对应空1、答案2对应空2；每个空可分别设置多个等价答案。</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>50||50赫兹</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>示例·简答（填好后删）简述输电线路巡视前应完成的主要安全准备。</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>简答</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>简答，安全，示例</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>示例解析：简答题由答题者对照参考答案自行判定正确或错误。</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>确认天气和现场风险，核对线路及作业信息，准备并检查必要的安全防护用品和巡视工具。</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -442,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>必填。支持普通文字、公式、【图1】等图片占位符，以及计算题的【空1】【空2】等填空占位符。</t>
+          <t>必填。支持普通文字、公式、【图1】等图片占位符，以及计算题/填空题的【空1】【空2】等答题占位符。</t>
         </is>
       </c>
     </row>
@@ -454,7 +504,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>必填，只能填写：单选、多选、判断、计算。</t>
+          <t>必填，只能填写：单选、多选、判断、计算、填空、简答。</t>
         </is>
       </c>
     </row>
@@ -466,7 +516,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>所有题至少填写答案1。单选、多选、判断只填写答案1；计算题按填空顺序分别填写答案1、答案2…，答案列之间不得留空。</t>
+          <t>模板只预留答案1、答案2两列。所有题至少填写答案1；单选、多选、判断、简答只填写答案1；计算题、填空题按空位顺序填写答案1、答案2……。如需更多空位，请在选项A之前继续插入答案3、答案4……，答案/填空最多 12 列，且答案列之间不得留空。</t>
         </is>
       </c>
     </row>
@@ -502,7 +552,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>单选、多选、判断题的选项从答案列右侧的 A 列开始连续填写，不得断列；判断题必须依次为“正确、错误”。计算题不要填写选项。</t>
+          <t>模板只预留 A、B、C、D 四列。只有单选、多选、判断题填写选项；需要更多选项时可在图片列之前继续按 E、F、G……连续增加。判断题必须依次为“正确、错误”。计算、填空、简答题不要填写选项。</t>
         </is>
       </c>
     </row>
@@ -533,58 +583,82 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>图片题</t>
+          <t>填空题</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>支持题干图片和选项图片。先在题干或选项文字中写【图1】【图2】等占位符，再把对应图片按编号放入本行末尾的“图片1”“图片2”列。每一题都从图1重新编号。</t>
+          <t>答案1对应第1空、答案2对应第2空……；同一空有多个可接受答案时，在同一个答案单元格内用 || 分隔，例如“电流||电流强度”。答案比较会忽略首尾空格并统一大小写/全半角。填空题不填写选项。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>插入图片</t>
+          <t>简答题</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>推荐使用 WPS 的“插入图片→嵌入单元格”，并保持图片列位于全部选项列之后且从“图片1”连续编号。不要填写本机路径或网络图片地址。</t>
+          <t>只填写答案1作为参考答案，其余答案列与全部选项列留空。练习时先作答，再对照参考答案自行判定正确或错误。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>兼容提示</t>
+          <t>图片题</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>模板图片采用 WPS DISPIMG 单元格图片格式；WPS 可正常查看和编辑。部分 Microsoft Excel 版本可能显示 #NAME?，但请勿删除图片列或公式，以免导入时丢图。</t>
+          <t>支持题干图片和选项图片。先在题干或选项文字中写【图1】【图2】等占位符，再把对应图片按编号放入本行末尾的“图片1”“图片2”列。每一题都从图1重新编号。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>限制</t>
+          <t>插入图片</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>单次最多导入 20,000 题；每题最多 12 个填空、24 个选项、12 张图片；Excel 文件最大 12 MB。</t>
+          <t>推荐使用 WPS 的“插入图片→嵌入单元格”，并保持图片列位于全部选项列之后且从“图片1”连续编号。不要填写本机路径或网络图片地址。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>兼容提示</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>模板图片继续使用原模板同一张拾卷图标，并采用 WPS DISPIMG 单元格图片格式；WPS 可正常查看和编辑。部分 Microsoft Excel 版本可能显示 #NAME?，但请勿删除图片列或公式，以免导入时丢图。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>限制</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>模板仅预留 2 个答案列和 4 个选项列；系统答案/填空上限为 12 列。需要更多列时按上述规则连续扩展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>安全提醒</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>图片会作为本地私有资产导入并随私有仓库同步；不要在工作簿中填写 GitHub 令牌或其他账号凭据。</t>
         </is>

</xml_diff>